<commit_message>
Expand Kahoot to 20 questions and retime the talk to stay at 40 minutes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -501,34 +501,34 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>¿Con qué tiene que terminar siempre una reunión con un cliente?</t>
+          <t>En Zent, ¿quién vende?</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Un siguiente paso: qué, quién y cuándo</t>
+          <t>Sólo el equipo comercial</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Una demo del agente</t>
+          <t>Sólo los socios</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>El precio del proyecto</t>
+          <t>Todo el equipo, también delivery</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Un café</t>
+          <t>Nadie, se vende solo</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -537,31 +537,23 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Experiencia = (producto + servicio) dividido por...</t>
+          <t>Verdadero o falso: que el gerente nos caiga bien significa que tiene intención de compra.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Precio + plazo</t>
+          <t>Verdadero</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Necesidad + deseo</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Horas + equipo</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Riesgo + costo</t>
-        </is>
-      </c>
+          <t>Falso</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>2</v>
@@ -573,27 +565,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Si vendemos magia, un agente que funciona bien igual se siente...</t>
+          <t>¿Cuál de estos NO es uno de los 6 errores comunes en B2B?</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Mayor a 1: wow</t>
+          <t>Hablar de la solución antes que del problema</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Igual a 1</t>
+          <t>Irse sin acordar el siguiente paso</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Menor a 1: decepción</t>
+          <t>Preguntar cuánto le cuesta hoy el problema</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>No se nota</t>
+          <t>Vender características, no resultados</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -609,34 +601,34 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Cuando un cliente contrata un agente de IA, ¿qué compra en realidad?</t>
+          <t>Experiencia = (producto + servicio) dividido por...</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Un modelo de lenguaje</t>
+          <t>Precio + plazo</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Horas de desarrollo</t>
+          <t>Necesidad + deseo</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Capacidad sin sumar estructura</t>
+          <t>Horas + equipo</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Un software</t>
+          <t>Riesgo + costo</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -645,34 +637,34 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>La gente compra cuando el costo de no hacer nada es...</t>
+          <t>Si vendemos magia, un agente que funciona bien igual se siente...</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Igual a cero</t>
+          <t>Mayor a 1: wow</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Mayor al costo de actuar</t>
+          <t>Igual a 1</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Menor al presupuesto</t>
+          <t>Menor a 1: decepción</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>No se nota</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -681,34 +673,34 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>En proyectos de IA, ¿quién suele ser el bloqueador típico?</t>
+          <t>En la decisión de compra, el sistema rápido decide. ¿Qué hace el sistema lento?</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Quien teme ser reemplazado</t>
+          <t>Firma</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>El gerente general</t>
+          <t>Justifica</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>El área de sistemas</t>
+          <t>Bloquea</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>El proveedor actual</t>
+          <t>Olvida</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -717,27 +709,27 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>¿Qué hacía Heineken con las notas de voz de más de 3 minutos?</t>
+          <t>¿Cuál de estos es un deseo emocional, no una conveniencia racional?</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Las transcribía con IA</t>
+          <t>Ahorrar horas de carga manual</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Las publicaba en redes</t>
+          <t>Reducir costos</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Las cambiaba por una cerveza para verse en persona</t>
+          <t>Ser quien modernizó la empresa</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Las borraba</t>
+          <t>Bajar la tasa de errores</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
@@ -753,33 +745,457 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>¿Cuál de estos es uno de los 5 drivers psicológicos de compra?</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Evitar un dolor o un temor</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>El color del logo</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>La cantidad de diapositivas</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>El stack técnico</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Cuando un cliente contrata un agente de IA, ¿qué compra en realidad?</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Un modelo de lenguaje</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Horas de desarrollo</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Capacidad sin sumar estructura</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Un software</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>En la fórmula de la propuesta de valor, ¿qué va después de "evitando..."?</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>El precio</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>El dolor principal</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>El nombre del cliente</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>La tecnología que usamos</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>En el mapa de poder del cliente, ¿quién tiene la autoridad y la firma?</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>El iniciador</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>El decisor</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>El beneficiario</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>El influenciador</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>En proyectos de IA, ¿quién suele ser el bloqueador típico?</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Quien teme ser reemplazado</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>El gerente general</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>El área de sistemas</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>El proveedor actual</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>¿En qué paso del proceso consultivo el cliente percibe la urgencia de actuar?</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Conectar</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Construir la solución</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Pasar a la acción</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Problematizar</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>La gente compra cuando el costo de no hacer nada es...</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Igual a cero</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Mayor al costo de actuar</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Menor al presupuesto</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>¿Qué pregunta de discovery sirve para definir el éxito del proyecto?</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>¿Cuánto presupuesto tienen?</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>¿Ya usan ChatGPT?</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>¿Qué tendrían que ver en 6 meses para decir que funcionó?</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>¿Cuándo firmamos?</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
           <t>Objeción: "Ya usamos ChatGPT". ¿Cuál es la mejor respuesta?</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Ofrecer un descuento</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Una herramienta no es un proceso adoptado, medido y mantenido</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Decir que ChatGPT es peor</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Entonces no nos necesitan</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="H11" s="3" t="n">
+      <c r="G19" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>¿Cuál de estos NO es uno de los 5 filtros de una propuesta que convence?</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Creíble</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Larga y detallada</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Emotiva</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>¿Qué hacía Heineken con las notas de voz de más de 3 minutos?</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Las transcribía con IA</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Las publicaba en redes</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Las cambiaba por una cerveza para verse en persona</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Las borraba</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Verdadero o falso: el social selling es 80% venta y 20% contenido.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Verdadero</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Falso</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>¿Cuál es uno de los tres compromisos para el lunes?</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Mandar más mails por semana</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Ninguna reunión termina sin siguiente paso</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Bajar los precios</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Hacer más demos</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H23" s="3" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use the original Sperry brain model wording on slide 7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -673,27 +673,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>En la decisión de compra, el sistema rápido decide. ¿Qué hace el sistema lento?</t>
+          <t>En el modelo de Roger Sperry, ¿qué lógica corresponde al hemisferio derecho?</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Firma</t>
+          <t>La lógica de la conveniencia</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Justifica</t>
+          <t>La lógica de la creencia</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Bloquea</t>
+          <t>La lógica secuencial</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Olvida</t>
+          <t>La lógica del precio</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">

</xml_diff>

<commit_message>
Remove discovery divider, power map and consultative process slides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -853,27 +853,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>En el mapa de poder del cliente, ¿quién tiene la autoridad y la firma?</t>
+          <t>Según el dato popular, ¿cuántos segundos de atención tiene una persona?</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>El iniciador</t>
+          <t>2 segundos</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>El decisor</t>
+          <t>8 segundos</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>El beneficiario</t>
+          <t>30 segundos</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>El influenciador</t>
+          <t>60 segundos</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
@@ -889,34 +889,34 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>En proyectos de IA, ¿quién suele ser el bloqueador típico?</t>
+          <t>Objeción: "Nuestros datos no están listos". ¿Qué respondemos?</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Quien teme ser reemplazado</t>
+          <t>Entonces no podemos trabajar</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>El gerente general</t>
+          <t>Que los ordene otro proveedor</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>El área de sistemas</t>
+          <t>Ordenarlos es parte de la etapa inicial</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>El proveedor actual</t>
+          <t>Esperar un año</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -925,34 +925,34 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>¿En qué paso del proceso consultivo el cliente percibe la urgencia de actuar?</t>
+          <t>¿Qué pregunta de discovery ayuda a medir el costo de no actuar?</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Conectar</t>
+          <t>Si esto sigue igual 12 meses, ¿qué les cuesta?</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Construir la solución</t>
+          <t>¿Qué herramienta usan?</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Pasar a la acción</t>
+          <t>¿Quién es su proveedor?</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Problematizar</t>
+          <t>¿Les gustó la demo?</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Remove experience-equation slide and update its Kahoot questions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -601,34 +601,34 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Experiencia = (producto + servicio) dividido por...</t>
+          <t>Según la diapositiva de los tres cerebros, ¿qué porcentaje de la decisión es emocional?</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Precio + plazo</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Necesidad + deseo</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Horas + equipo</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Riesgo + costo</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -637,34 +637,34 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Si vendemos magia, un agente que funciona bien igual se siente...</t>
+          <t>En B2B, ¿cuál de estos es un deseo emocional del cliente?</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Mayor a 1: wow</t>
+          <t>El precio más bajo</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Igual a 1</t>
+          <t>Gestión fácil: no quiero transpirar</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Menor a 1: decepción</t>
+          <t>Más funcionalidades</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>No se nota</t>
+          <t>Un contrato más largo</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Remove slides 30-34 (impact, visibility block and commitments)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Verdadero o falso: el social selling es 80% venta y 20% contenido.</t>
+          <t>Verdadero o falso: en el caso de The Economist, la opción "sólo impresa" estaba para que nadie la eligiera.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1160,7 +1160,7 @@
         <v>10</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1169,27 +1169,27 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>¿Cuál es uno de los tres compromisos para el lunes?</t>
+          <t>Según el anclaje de precios, ¿qué conviene mostrar antes que nuestro precio?</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Mandar más mails por semana</t>
+          <t>Un descuento</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Ninguna reunión termina sin siguiente paso</t>
+          <t>El costo del problema para el cliente</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Bajar los precios</t>
+          <t>La opción más barata</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Hacer más demos</t>
+          <t>El stack técnico</t>
         </is>
       </c>
       <c r="G23" s="3" t="n">

</xml_diff>

<commit_message>
Remove agenda, 'todos vendemos' and B2B errors slides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -501,34 +501,34 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>En Zent, ¿quién vende?</t>
+          <t>Según la charla, ¿qué dispara la decisión de compra?</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Sólo el equipo comercial</t>
+          <t>Los números</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Sólo los socios</t>
+          <t>La confianza y el deseo</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Todo el equipo, también delivery</t>
+          <t>El precio más bajo</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Nadie, se vende solo</t>
+          <t>La tecnología</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -537,23 +537,31 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Verdadero o falso: que el gerente nos caiga bien significa que tiene intención de compra.</t>
+          <t>Según la curva de atención, ¿cuánta audiencia se pierde a los 10 minutos?</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Verdadero</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Falso</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>2</v>
@@ -565,27 +573,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>¿Cuál de estos NO es uno de los 6 errores comunes en B2B?</t>
+          <t>¿Qué recupera la atención durante una charla o una demo?</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Hablar de la solución antes que del problema</t>
+          <t>Más diapositivas</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Irse sin acordar el siguiente paso</t>
+          <t>Hablar más rápido</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Preguntar cuánto le cuesta hoy el problema</t>
+          <t>Una broma, una historia o una pregunta</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Vender características, no resultados</t>
+          <t>Bajar las luces</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">

</xml_diff>

<commit_message>
Rebuild 20-question Kahoot from the current talk and Heineken video
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2sePAHLe9D4GCAzGMXE7H
</commit_message>
<xml_diff>
--- a/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
+++ b/charlas/como-vendemos-en-zent/kahoot-preguntas.xlsx
@@ -501,27 +501,27 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Según la charla, ¿qué dispara la decisión de compra?</t>
+          <t>En el modelo de los hemisferios, el hemisferio izquierdo responde a la lógica de...</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Los números</t>
+          <t>La creencia</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>La confianza y el deseo</t>
+          <t>La conveniencia</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>El precio más bajo</t>
+          <t>El deseo</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>La tecnología</t>
+          <t>La intuición</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -537,34 +537,34 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Según la curva de atención, ¿cuánta audiencia se pierde a los 10 minutos?</t>
+          <t>Según la diapositiva de los tres cerebros, ¿qué porcentaje de la decisión es emocional?</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -573,27 +573,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>¿Qué recupera la atención durante una charla o una demo?</t>
+          <t>¿Qué cerebro se encarga del instinto: sobrevivir, reaccionar, respirar?</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Más diapositivas</t>
+          <t>El límbico</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Hablar más rápido</t>
+          <t>El neocórtex</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Una broma, una historia o una pregunta</t>
+          <t>El reptiliano</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Bajar las luces</t>
+          <t>El cortical</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -609,34 +609,26 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Según la diapositiva de los tres cerebros, ¿qué porcentaje de la decisión es emocional?</t>
+          <t>Verdadero o falso: somos seres racionales que sienten.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Verdadero</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>85%</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
+          <t>Falso</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -681,27 +673,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>En el modelo de Roger Sperry, ¿qué lógica corresponde al hemisferio derecho?</t>
+          <t>Según la charla, ¿qué dispara la decisión de compra?</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>La lógica de la conveniencia</t>
+          <t>Los números</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>La lógica de la creencia</t>
+          <t>La confianza y el deseo</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>La lógica secuencial</t>
+          <t>El precio más bajo</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>La lógica del precio</t>
+          <t>La tecnología</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
@@ -717,34 +709,34 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>¿Cuál de estos es un deseo emocional, no una conveniencia racional?</t>
+          <t>¿Cuál de estos es uno de los 5 drivers psicológicos de compra?</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Ahorrar horas de carga manual</t>
+          <t>Evitar un dolor o un temor</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Reducir costos</t>
+          <t>El color del logo</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Ser quien modernizó la empresa</t>
+          <t>La cantidad de diapositivas</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Bajar la tasa de errores</t>
+          <t>El stack técnico</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -753,34 +745,34 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>¿Cuál de estos es uno de los 5 drivers psicológicos de compra?</t>
+          <t>Cuando un cliente contrata un agente de IA, ¿qué compra en realidad?</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Evitar un dolor o un temor</t>
+          <t>Un modelo de lenguaje</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>El color del logo</t>
+          <t>Horas de desarrollo</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>La cantidad de diapositivas</t>
+          <t>Capacidad sin sumar estructura</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>El stack técnico</t>
+          <t>Un software</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -789,34 +781,34 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cuando un cliente contrata un agente de IA, ¿qué compra en realidad?</t>
+          <t>En la fórmula de la propuesta de valor, ¿qué va después de "evitando..."?</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Un modelo de lenguaje</t>
+          <t>El precio</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Horas de desarrollo</t>
+          <t>El dolor principal</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Capacidad sin sumar estructura</t>
+          <t>El nombre del cliente</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Un software</t>
+          <t>La tecnología que usamos</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -825,27 +817,27 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>En la fórmula de la propuesta de valor, ¿qué va después de "evitando..."?</t>
+          <t>La gente compra cuando el costo de no hacer nada es...</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>El precio</t>
+          <t>Igual a cero</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>El dolor principal</t>
+          <t>Mayor al costo de actuar</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>El nombre del cliente</t>
+          <t>Menor al presupuesto</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>La tecnología que usamos</t>
+          <t>Desconocido</t>
         </is>
       </c>
       <c r="G13" s="3" t="n">
@@ -861,34 +853,34 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Según el dato popular, ¿cuántos segundos de atención tiene una persona?</t>
+          <t>En el caso de The Economist, ¿qué porcentaje eligió impresa + web?</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2 segundos</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>8 segundos</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>30 segundos</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>60 segundos</t>
+          <t>84%</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -897,34 +889,34 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Objeción: "Nuestros datos no están listos". ¿Qué respondemos?</t>
+          <t>¿Para qué estaba la opción "sólo impresa" a US$ 125?</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Entonces no podemos trabajar</t>
+          <t>Para vender más revistas en papel</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Que los ordene otro proveedor</t>
+          <t>Para que la opción completa pareciera un regalo</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Ordenarlos es parte de la etapa inicial</t>
+          <t>Fue un error de imprenta</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Esperar un año</t>
+          <t>Para bajar costos</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -933,34 +925,34 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>¿Qué pregunta de discovery ayuda a medir el costo de no actuar?</t>
+          <t>En el experimento del teclado, ¿qué número funcionó como ancla?</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Si esto sigue igual 12 meses, ¿qué les cuesta?</t>
+          <t>El precio de mercado</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>¿Qué herramienta usan?</t>
+          <t>La edad de cada uno</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>¿Quién es su proveedor?</t>
+          <t>Los dos últimos dígitos del documento</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>¿Les gustó la demo?</t>
+          <t>Un número sorteado</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -969,27 +961,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>La gente compra cuando el costo de no hacer nada es...</t>
+          <t>Según el anclaje de precios, ¿qué conviene mostrar antes que nuestro precio?</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Igual a cero</t>
+          <t>Un descuento</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Mayor al costo de actuar</t>
+          <t>El costo del problema para el cliente</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Menor al presupuesto</t>
+          <t>La opción más barata</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>El stack técnico</t>
         </is>
       </c>
       <c r="G17" s="3" t="n">
@@ -1005,34 +997,34 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>¿Qué pregunta de discovery sirve para definir el éxito del proyecto?</t>
+          <t>Objeción: "Ya usamos ChatGPT". ¿Cuál es la mejor respuesta?</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>¿Cuánto presupuesto tienen?</t>
+          <t>Ofrecer un descuento</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>¿Ya usan ChatGPT?</t>
+          <t>Una herramienta no es un proceso adoptado, medido y mantenido</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>¿Qué tendrían que ver en 6 meses para decir que funcionó?</t>
+          <t>Decir que ChatGPT es peor</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo firmamos?</t>
+          <t>Entonces no nos necesitan</t>
         </is>
       </c>
       <c r="G18" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1041,27 +1033,27 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Objeción: "Ya usamos ChatGPT". ¿Cuál es la mejor respuesta?</t>
+          <t>Según la curva de atención, ¿cuánta audiencia se pierde a los 10 minutos?</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Ofrecer un descuento</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Una herramienta no es un proceso adoptado, medido y mantenido</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Decir que ChatGPT es peor</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Entonces no nos necesitan</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="G19" s="3" t="n">
@@ -1077,34 +1069,34 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>¿Cuál de estos NO es uno de los 5 filtros de una propuesta que convence?</t>
+          <t>Video de Heineken: ¿qué tenías que reenviarle por WhatsApp?</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Una foto en un bar</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Creíble</t>
+          <t>Una nota de voz de más de 3 minutos</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Larga y detallada</t>
+          <t>Un meme</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Emotiva</t>
+          <t>Tu documento</t>
         </is>
       </c>
       <c r="G20" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -1113,27 +1105,27 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>¿Qué hacía Heineken con las notas de voz de más de 3 minutos?</t>
+          <t>Video de Heineken: ¿qué recibías a cambio?</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Las transcribía con IA</t>
+          <t>Un descuento en datos móviles</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Las publicaba en redes</t>
+          <t>Un sticker</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Las cambiaba por una cerveza para verse en persona</t>
+          <t>Un cupón de cerveza y bares cerca para juntarte en persona</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Las borraba</t>
+          <t>Una gorra</t>
         </is>
       </c>
       <c r="G21" s="3" t="n">
@@ -1149,26 +1141,34 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Verdadero o falso: en el caso de The Economist, la opción "sólo impresa" estaba para que nadie la eligiera.</t>
+          <t>Video de Heineken: ¿en qué país se lanzó la campaña?</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Verdadero</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Falso</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Holanda</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
       <c r="G22" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -1177,27 +1177,27 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Según el anclaje de precios, ¿qué conviene mostrar antes que nuestro precio?</t>
+          <t>Video de Heineken: ¿qué insight usó la marca?</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Un descuento</t>
+          <t>La gente toma menos cerveza</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>El costo del problema para el cliente</t>
+          <t>Las notas de voz largas reemplazan los encuentros reales</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>La opción más barata</t>
+          <t>WhatsApp es aburrido</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>El stack técnico</t>
+          <t>Nadie escucha audios</t>
         </is>
       </c>
       <c r="G23" s="3" t="n">

</xml_diff>